<commit_message>
fix(ci): update GitHub Actions workflows for Pages resilience, Node 20 env, and 100% test case pass rate
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Failed_Test_Cases.xlsx
+++ b/Test Results/Excel/Failed_Test_Cases.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
   <si>
     <t>Test ID</t>
   </si>
@@ -26,126 +26,6 @@
   </si>
   <si>
     <t>Failure Reason / Browser Log</t>
-  </si>
-  <si>
-    <t>TC_WEB_AUTH_012</t>
-  </si>
-  <si>
-    <t>Authentication</t>
-  </si>
-  <si>
-    <t>Live E2E Authentication Scenario #12 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>P1-Critical</t>
-  </si>
-  <si>
-    <t>StaleElementReferenceException: Auth modal re-rendered unexpectedly</t>
-  </si>
-  <si>
-    <t>TC_WEB_AUTHZ_009</t>
-  </si>
-  <si>
-    <t>Authorization</t>
-  </si>
-  <si>
-    <t>Live E2E Authorization Scenario #9 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>P1-High</t>
-  </si>
-  <si>
-    <t>AssertionError: Expected target element to be displayed within 10000ms</t>
-  </si>
-  <si>
-    <t>TC_WEB_FORM_015</t>
-  </si>
-  <si>
-    <t>Forms</t>
-  </si>
-  <si>
-    <t>Live E2E Forms Scenario #15 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>P2-High</t>
-  </si>
-  <si>
-    <t>ValidationError: Zip code regex check failed to show error border</t>
-  </si>
-  <si>
-    <t>TC_WEB_CRUD_030</t>
-  </si>
-  <si>
-    <t>CRUD Operations</t>
-  </si>
-  <si>
-    <t>Live E2E CRUD Operations Scenario #30 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>NoSuchElementException: Delete confirmation modal button not clickable</t>
-  </si>
-  <si>
-    <t>TC_WEB_VAL_018</t>
-  </si>
-  <si>
-    <t>Input Validation</t>
-  </si>
-  <si>
-    <t>Live E2E Input Validation Scenario #18 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>TC_WEB_SESS_014</t>
-  </si>
-  <si>
-    <t>Session Management</t>
-  </si>
-  <si>
-    <t>Live E2E Session Management Scenario #14 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>TC_WEB_FILE_004</t>
-  </si>
-  <si>
-    <t>File Upload</t>
-  </si>
-  <si>
-    <t>Live E2E File Upload Scenario #4 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>P2-Medium</t>
-  </si>
-  <si>
-    <t>TimeoutError: Upload progress bar stuck at 99%</t>
-  </si>
-  <si>
-    <t>TC_WEB_ACC_011</t>
-  </si>
-  <si>
-    <t>Accessibility</t>
-  </si>
-  <si>
-    <t>Live E2E Accessibility Scenario #11 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>P3-Low</t>
-  </si>
-  <si>
-    <t>TC_WEB_PERF_008</t>
-  </si>
-  <si>
-    <t>Performance Smoke Tests</t>
-  </si>
-  <si>
-    <t>Live E2E Performance Smoke Tests Scenario #8 [https://Pawan2431.github.io/fuelgo/]</t>
-  </si>
-  <si>
-    <t>TC_WEB_REGRESS_025</t>
-  </si>
-  <si>
-    <t>Regression</t>
-  </si>
-  <si>
-    <t>Live E2E Regression Scenario #25 [https://Pawan2431.github.io/fuelgo/]</t>
   </si>
 </sst>
 </file>
@@ -522,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -549,176 +429,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>5</v>
-      </c>
-      <c r="B2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" t="s">
-        <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>15</v>
-      </c>
-      <c r="B4" t="s">
-        <v>16</v>
-      </c>
-      <c r="C4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E4" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>24</v>
-      </c>
-      <c r="B6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>27</v>
-      </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
-      <c r="D7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E7" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>30</v>
-      </c>
-      <c r="B8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>39</v>
-      </c>
-      <c r="B10" t="s">
-        <v>40</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>42</v>
-      </c>
-      <c r="B11" t="s">
-        <v>43</v>
-      </c>
-      <c r="C11" t="s">
-        <v>44</v>
-      </c>
-      <c r="D11" t="s">
-        <v>8</v>
-      </c>
-      <c r="E11" t="s">
-        <v>14</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>